<commit_message>
feat: finalize evaluation and index integrity fixes
</commit_message>
<xml_diff>
--- a/data/eval/QA数据.xlsx
+++ b/data/eval/QA数据.xlsx
@@ -1223,10 +1223,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O301"/>
+  <dimension ref="A1:P301"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.3846153846154" defaultRowHeight="16.8"/>
   <cols>
     <col width="43.75" customWidth="1" style="1" min="15" max="15"/>
+    <col width="20" customWidth="1" style="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1305,6 +1306,11 @@
           <t>file_label</t>
         </is>
       </c>
+      <c r="P1" s="0" t="inlineStr">
+        <is>
+          <t>eval_status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
@@ -6658,6 +6664,11 @@
       <c r="O76" s="0" t="inlineStr">
         <is>
           <t>银行业金融机构资产负债情况表(季度).xlsx</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>excluded_ambiguous</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: finalize competition evaluation and table retrieval
</commit_message>
<xml_diff>
--- a/data/eval/QA数据.xlsx
+++ b/data/eval/QA数据.xlsx
@@ -2546,7 +2546,7 @@
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>根据 Excel 附件《2023年商业银行主要监管指标情况表（季度）》（工作表：商业银行季度），“正常类贷款”在“季度”口径下的数值是多少？</t>
+          <t>根据 Excel 附件《2023年商业银行主要监管指标情况表（季度）》（工作表：商业银行季度），“正常类贷款”在“一季度”口径下的数值是多少？</t>
         </is>
       </c>
       <c r="G20" s="0" t="n">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>根据 Excel 附件《2023年银行业总资产、总负债（季度）》（工作表：资产负债季度），“总资产”在“年-季度”口径下的数值是多少？</t>
+          <t>根据 Excel 附件《2023年银行业总资产、总负债（季度）》（工作表：资产负债季度），“总资产”在“一季度”口径下的数值是多少？</t>
         </is>
       </c>
       <c r="G21" s="0" t="n">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>根据 Excel 附件《2023年银行业金融机构保障性安居工程贷款情况表(季度)》（工作表： 保障房贷款），“银行业金融机构合计”在“年-季度”口径下的数值是多少？</t>
+          <t>根据 Excel 附件《2023年银行业金融机构保障性安居工程贷款情况表(季度)》（工作表： 保障房贷款），“银行业金融机构合计”在“一季度”口径下的数值是多少？</t>
         </is>
       </c>
       <c r="G22" s="0" t="n">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>根据 Excel 附件《2023年银行业金融机构普惠型小微企业贷款情况（季度）》（工作表：普惠型小微企业贷款），“银行业金融机构合计”在“年-季度”口径下的数值是多少？</t>
+          <t>根据 Excel 附件《2023年银行业金融机构普惠型小微企业贷款情况（季度）》（工作表：普惠型小微企业贷款），“银行业金融机构合计”在“一季度”口径下的数值是多少？</t>
         </is>
       </c>
       <c r="G23" s="0" t="n">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>根据 Excel 附件《2023年银行业金融机构保障性安居工程贷款情况表(季度)》（工作表： 保障房贷款），在“年-季度”口径下，以下哪一项数值最高？</t>
+          <t>根据 Excel 附件《2023年银行业金融机构保障性安居工程贷款情况表(季度)》（工作表： 保障房贷款），在“一季度”口径下，以下哪一项数值最高？</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>根据 Excel 附件《2023年银行业金融机构普惠型小微企业贷款情况（季度）》（工作表：普惠型小微企业贷款），在“年-季度”口径下，以下哪一项数值最高？</t>
+          <t>根据 Excel 附件《2023年银行业金融机构普惠型小微企业贷款情况（季度）》（工作表：普惠型小微企业贷款），在“一季度”口径下，以下哪一项数值最高？</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
@@ -4875,17 +4875,17 @@
       </c>
       <c r="K52" s="0" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="L52" s="0" t="inlineStr">
         <is>
-          <t>原保险保费收入</t>
+          <t>保险金额</t>
         </is>
       </c>
       <c r="M52" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/091_2024年9月财产保险公司经营情况表_2024年9月财产险公司经营情况表.xlsx；工作表：产险公司数据（月度）  ；单位:亿元；原保险保费收入=13066.56(C7)；机动车辆保险=6545.53(C8)；责任险=1097.52(C9)；农业保险=1371.38(C10)；健康险=1818.56(C11)；意外险=403.31(C12)。</t>
+          <t>data/raw/nfra_page_attachments_500/091_2024年9月财产保险公司经营情况表_2024年9月财产险公司经营情况表.xlsx；工作表：产险公司数据（月度）  ；单位:亿元；责任险=1097.52(C9)；原保险保费收入=13066.56(C7)；机动车辆保险=6545.53(C8)；保险金额=125426586.62(C14)。</t>
         </is>
       </c>
       <c r="N52" s="0" t="inlineStr">
@@ -4952,17 +4952,17 @@
       </c>
       <c r="K53" s="0" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L53" s="0" t="inlineStr">
         <is>
-          <t>原保险保费收入</t>
+          <t>新增保险金额</t>
         </is>
       </c>
       <c r="M53" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/057_2025年3月人身险公司经营情况表_2025年3月人身险公司经营情况表.xlsx；工作表：人身保险公司（月度）  ；单位:亿元；原保险保费收入=16590.18(C6)；寿险=13832.14(C7)；意外险=117.14(C8)；健康险=2640.91(C9)；保户投资款新增交费=2605.25(C10)；投连险独立账户新增交费=33.83(C11)。</t>
+          <t>data/raw/nfra_page_attachments_500/057_2025年3月人身险公司经营情况表_2025年3月人身险公司经营情况表.xlsx；工作表：人身保险公司（月度）  ；单位:亿元；新增保险金额=3816438.23(C13)；寿险=13832.14(C7)；原保险保费收入=16590.18(C6)；意外险=117.14(C8)。</t>
         </is>
       </c>
       <c r="N53" s="0" t="inlineStr">
@@ -5029,17 +5029,17 @@
       </c>
       <c r="K54" s="0" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L54" s="0" t="inlineStr">
         <is>
-          <t>原保险保费收入</t>
+          <t>总资产</t>
         </is>
       </c>
       <c r="M54" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/059_2025年3月保险业经营情况表_2025年3月保险业经营情况表.xlsx；工作表：保险业经营数据（月度）；单位:亿元；原保险保费收入=21745(C6)；财产险=3867(C7)；人身险=17878(C8)；原保险赔付支出=8273.6(C9)；财产险=2124.55(C10)；人身险=6149.05(C11)。</t>
+          <t>data/raw/nfra_page_attachments_500/059_2025年3月保险业经营情况表_2025年3月保险业经营情况表.xlsx；工作表：保险业经营数据（月度）；单位:亿元；财产险=3867(C7)；人身险=17878(C8)；总资产=378425.19(C12)；原保险保费收入=21745(C6)。</t>
         </is>
       </c>
       <c r="N54" s="0" t="inlineStr">
@@ -5491,17 +5491,17 @@
       </c>
       <c r="K60" s="0" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L60" s="0" t="inlineStr">
         <is>
-          <t>原保险保费收入</t>
+          <t>保险金额</t>
         </is>
       </c>
       <c r="M60" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/058_2025年3月财产保险公司经营情况表_2025年3月财产险公司经营情况表.xlsx；工作表：产险公司数据（月度）  ；单位:亿元；原保险保费收入=5155(C7)；机动车辆保险=2234.09(C8)；责任险=425.49(C9)；农业保险=455.23(C10)；健康险=1140.9(C11)；意外险=147.48(C12)。</t>
+          <t>data/raw/nfra_page_attachments_500/058_2025年3月财产保险公司经营情况表_2025年3月财产险公司经营情况表.xlsx；工作表：产险公司数据（月度）  ；单位:亿元；保险金额=45933310.37(C14)；机动车辆保险=2234.09(C8)；责任险=425.49(C9)；原保险保费收入=5155(C7)。</t>
         </is>
       </c>
       <c r="N60" s="0" t="inlineStr">
@@ -5568,17 +5568,17 @@
       </c>
       <c r="K61" s="0" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="L61" s="0" t="inlineStr">
         <is>
-          <t>原保险保费收入</t>
+          <t>新增保险金额</t>
         </is>
       </c>
       <c r="M61" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/033_2025年9月人身险公司经营情况表_2025年9月人身险公司经营情况表.xlsx；工作表：人身保险公司（月度）  ；单位:亿元；原保险保费收入=38433.67(C5)；寿险=31707.74(C6)；意外险=304.39(C7)；健康险=6421.53(C8)；保户投资款新增交费=5032.08(C9)；投连险独立账户新增交费=167.34(C10)。</t>
+          <t>data/raw/nfra_page_attachments_500/033_2025年9月人身险公司经营情况表_2025年9月人身险公司经营情况表.xlsx；工作表：人身保险公司（月度）  ；单位:亿元；意外险=304.39(C7)；新增保险金额=8740661.75(C12)；寿险=31707.74(C6)；原保险保费收入=38433.67(C5)。</t>
         </is>
       </c>
       <c r="N61" s="0" t="inlineStr">
@@ -5645,17 +5645,17 @@
       </c>
       <c r="K62" s="0" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L62" s="0" t="inlineStr">
         <is>
-          <t>原保险保费收入</t>
+          <t>总资产</t>
         </is>
       </c>
       <c r="M62" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/035_2025年9月保险业经营情况表_2025年9月保险业经营情况表.xlsx；工作表：保险业经营数据（月度）；单位:亿元；原保险保费收入=52145.77(C7)；财产险=11250.32(C8)；人身险=40895.45(C9)；赔付支出=18706.77(C10)；财产险=6981.4(C11)；人身险=11725.37(C12)。</t>
+          <t>data/raw/nfra_page_attachments_500/035_2025年9月保险业经营情况表_2025年9月保险业经营情况表.xlsx；工作表：保险业经营数据（月度）；单位:亿元；人身险=40895.45(C9)；原保险保费收入=52145.77(C7)；总资产=404005.89(C13)；财产险=11250.32(C8)。</t>
         </is>
       </c>
       <c r="N62" s="0" t="inlineStr">
@@ -6107,17 +6107,17 @@
       </c>
       <c r="K68" s="0" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="L68" s="0" t="inlineStr">
         <is>
-          <t>原保险保费收入</t>
+          <t>保险金额</t>
         </is>
       </c>
       <c r="M68" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/034_2025年9月财产保险公司经营情况表_2025年9月财产险公司经营情况表.xlsx；工作表：产险公司数据（月度）  ；单位:亿元；原保险保费收入=13712.1(C7)；机动车辆保险=6835.96(C8)；责任险=1148(C9)；农业保险=1410.17(C10)；健康险=2005.46(C11)；意外险=456.32(C12)。</t>
+          <t>data/raw/nfra_page_attachments_500/034_2025年9月财产保险公司经营情况表_2025年9月财产险公司经营情况表.xlsx；工作表：产险公司数据（月度）  ；单位:亿元；原保险保费收入=13712.1(C7)；机动车辆保险=6835.96(C8)；保险金额=138937806.41(C14)；责任险=1148(C9)。</t>
         </is>
       </c>
       <c r="N68" s="0" t="inlineStr">
@@ -6666,7 +6666,7 @@
           <t>银行业金融机构资产负债情况表(季度).xlsx</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr">
+      <c r="P76" s="0" t="inlineStr">
         <is>
           <t>excluded_ambiguous</t>
         </is>
@@ -6901,32 +6901,32 @@
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构保障性安居工程贷款情况表(季度)》，“股份制商业银行”从“年-季度”到“本年累计/截至当期”的数值变化约为多少？</t>
+          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构保障性安居工程贷款情况表(季度)》，“股份制商业银行”从“一季度”到“四季度”的数值变化约为多少？</t>
         </is>
       </c>
       <c r="G80" s="0" t="n">
-        <v>-5102.53</v>
+        <v>-295.18</v>
       </c>
       <c r="H80" s="0" t="n">
-        <v>-6236.43</v>
+        <v>-99.41</v>
       </c>
       <c r="I80" s="0" t="n">
-        <v>5669.48</v>
+        <v>-302.37</v>
       </c>
       <c r="J80" s="0" t="n">
-        <v>-5669.48</v>
+        <v>295.18</v>
       </c>
       <c r="K80" s="0" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L80" s="0" t="n">
-        <v>-5669.48</v>
+        <v>-295.18</v>
       </c>
       <c r="M80" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/132_2023年银行业金融机构保障性安居工程贷款情况表(季度)_银行业金融机构保障性安居工程贷款情况表(季度).xlsx；工作表： 保障房贷款；年-季度=5672.01(B8)，本年累计/截至当期=2.5261(J8)；变化值=-5669.48。</t>
+          <t>data/raw/nfra_page_attachments_500/132_2023年银行业金融机构保障性安居工程贷款情况表(季度)_银行业金融机构保障性安居工程贷款情况表(季度).xlsx；工作表： 保障房贷款；一季度=5672.01(B8)，四季度=5376.83(E8)；变化值=-295.18。</t>
         </is>
       </c>
       <c r="N80" s="0" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构保障性安居工程贷款情况表(季度)》，“银行业金融机构合计”从“年-季度”到“季度”的数值变化约为多少？</t>
+          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构保障性安居工程贷款情况表(季度)》，“银行业金融机构合计”从“一季度”到“四季度”的数值变化约为多少？</t>
         </is>
       </c>
       <c r="G81" s="0" t="n">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“农村金融机构”从“年-季度”到“季度”的数值变化约为多少？</t>
+          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“农村金融机构”从“一季度”到“四季度”的数值变化约为多少？</t>
         </is>
       </c>
       <c r="G82" s="0" t="n">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“城市商业银行”从“年-季度”到“季度”的数值变化约为多少？</t>
+          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“城市商业银行”从“一季度”到“四季度”的数值变化约为多少？</t>
         </is>
       </c>
       <c r="G83" s="0" t="n">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“大型商业银行”从“年-季度”到“季度”的数值变化约为多少？</t>
+          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“大型商业银行”从“一季度”到“四季度”的数值变化约为多少？</t>
         </is>
       </c>
       <c r="G84" s="0" t="n">
@@ -7236,32 +7236,32 @@
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“股份制商业银行”从“年-季度”到“本年累计/截至当期”的数值变化约为多少？</t>
+          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“股份制商业银行”从“一季度”到“四季度”的数值变化约为多少？</t>
         </is>
       </c>
       <c r="G85" s="0" t="n">
-        <v>-47197.64</v>
+        <v>1604.58</v>
       </c>
       <c r="H85" s="0" t="n">
-        <v>-42906.94</v>
+        <v>2866.18</v>
       </c>
       <c r="I85" s="0" t="n">
-        <v>-38616.25</v>
+        <v>-3733</v>
       </c>
       <c r="J85" s="0" t="n">
-        <v>42906.94</v>
+        <v>3733</v>
       </c>
       <c r="K85" s="0" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="L85" s="0" t="n">
-        <v>-42906.94</v>
+        <v>3733</v>
       </c>
       <c r="M85" s="0" t="inlineStr">
         <is>
-          <t>data/raw/nfra_page_attachments_500/131_2023年银行业金融机构普惠型小微企业贷款情况（季度）_银行业金融机构普惠型小微企业贷款情况表(季度).xlsx；工作表：普惠型小微企业贷款；年-季度=42909.43(B7)，本年累计/截至当期=2.4823(J7)；变化值=-42906.94。</t>
+          <t>data/raw/nfra_page_attachments_500/131_2023年银行业金融机构普惠型小微企业贷款情况（季度）_银行业金融机构普惠型小微企业贷款情况表(季度).xlsx；工作表：普惠型小微企业贷款；一季度=42909.43(B7)，四季度=46642.43(E7)；变化值=3733.00。</t>
         </is>
       </c>
       <c r="N85" s="0" t="inlineStr">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“银行业金融机构合计”从“年-季度”到“季度”的数值变化约为多少？</t>
+          <t>需要对同一 Excel 附件做两处取数并计算。根据《2023年银行业金融机构普惠型小微企业贷款情况（季度）》，“银行业金融机构合计”从“一季度”到“四季度”的数值变化约为多少？</t>
         </is>
       </c>
       <c r="G86" s="0" t="n">

</xml_diff>